<commit_message>
sort out Table2, 3
</commit_message>
<xml_diff>
--- a/dataset/CISB-dataset-detailed-info.xlsx
+++ b/dataset/CISB-dataset-detailed-info.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\cisb++\classification\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\suiren\CISB-dataset-main\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9A6E63-244D-4AF6-8F96-A423BDA6E1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B24E35F-74AF-4560-8592-97EAD8394594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5175" yWindow="4965" windowWidth="22815" windowHeight="16920" xr2:uid="{6F3C42E5-73A3-46E8-B7A0-530C32DFC8D8}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="31950" windowHeight="16920" xr2:uid="{6F3C42E5-73A3-46E8-B7A0-530C32DFC8D8}"/>
   </bookViews>
   <sheets>
     <sheet name="CISB-dataset-detailed-info" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="388">
   <si>
     <t>Unique bug id</t>
   </si>
@@ -561,145 +561,22 @@
     <t>a9d57ef15cbe327fe54416dd194ee0ea66ae53a4</t>
   </si>
   <si>
-    <t>reordering read</t>
-  </si>
-  <si>
-    <t>bf227a4f0558320513b86c279996021480f9e750</t>
-  </si>
-  <si>
-    <t>any</t>
-  </si>
-  <si>
-    <t>Ptr's volatile might be dropped by low version GCC. Use READ_ONCE to force volatile.</t>
-  </si>
-  <si>
-    <t>a6965b31888501f889261a6783f0de6afff84f8d</t>
-  </si>
-  <si>
-    <t>normal data race</t>
-  </si>
-  <si>
-    <t>data race-&gt;out of bound</t>
-  </si>
-  <si>
     <t>63a8dfb889112ab4a065aa60a9a1b590b410d055</t>
   </si>
   <si>
-    <t>NULL ptr dereference</t>
-  </si>
-  <si>
-    <t>load/store-&gt;race</t>
-  </si>
-  <si>
     <t>c1c0ce31b2420d5c173228a2132a492ede03d81f</t>
   </si>
   <si>
-    <t>tearing logic</t>
-  </si>
-  <si>
-    <t>f97eee484e71890131f9c563c5cc6d5a69e4308d</t>
-  </si>
-  <si>
-    <t>load tearing</t>
-  </si>
-  <si>
     <t>f2c3037811381f9149243828c7eb9a1631df9f9c</t>
   </si>
   <si>
-    <t>tearing logic load/store</t>
-  </si>
-  <si>
-    <t>eliminate bound check</t>
-  </si>
-  <si>
-    <t>ecabac70ff919580324b407818ee3e6c0004dcf8</t>
-  </si>
-  <si>
-    <t>check fail</t>
-  </si>
-  <si>
-    <t>add barrier_var</t>
-  </si>
-  <si>
     <t>49f683b41f28918df3e51ddc0d928cb2e934ccdb</t>
   </si>
   <si>
-    <t>l-4b</t>
-  </si>
-  <si>
-    <t>UB NULL ptr write</t>
-  </si>
-  <si>
     <t>7ded842b356d151ece8ac4985940438e6d3998bb</t>
   </si>
   <si>
-    <t>gcc reorders memcpy after an assignment because alias analysis thinks dst and assignment's lhs are on different objects. But in turn violates C standard of ptr arithmetic. In C's view, bpf_plt_ret and bpf_plt are distinct objects so cannot be subtracted. So alias fails.</t>
-  </si>
-  <si>
-    <t>l-26</t>
-  </si>
-  <si>
-    <t>env:_start failure</t>
-  </si>
-  <si>
-    <t>bff60150f7c464d80d86f289c056c2ad2afb3c05</t>
-  </si>
-  <si>
-    <t>When combined with -O0, -fomit-frame-pointer is defeated</t>
-  </si>
-  <si>
-    <t>l-7</t>
-  </si>
-  <si>
-    <t>CFI failure</t>
-  </si>
-  <si>
-    <t>ddf56288eebd1fe82c46fc9f693b5b18045cddb6</t>
-  </si>
-  <si>
-    <t>introducing insecure indirect call</t>
-  </si>
-  <si>
-    <t>discard</t>
-  </si>
-  <si>
-    <t>f0842bb3d38863777e3454da5653d80b5fde6321</t>
-  </si>
-  <si>
-    <t>Preventive. Add READ/WRITE_ONCe to avoid load fusing.</t>
-  </si>
-  <si>
-    <t>env:built-in replace</t>
-  </si>
-  <si>
-    <t>3f301dc292eb122eff61b8b2906e519154b0327f</t>
-  </si>
-  <si>
-    <t>replace --ffreestanding with finer-grained -fno-builtin</t>
-  </si>
-  <si>
-    <t>UB NULL ptr dereference</t>
-  </si>
-  <si>
     <t>b7cf07586c40f926063d4d09f7de28ff82f62b2a</t>
-  </si>
-  <si>
-    <t>memory barrier to forbid reordering</t>
-  </si>
-  <si>
-    <t>c3062ede9927053754ba27b280afe00b9b31b37a</t>
-  </si>
-  <si>
-    <t>load tearing. Accessing volatile with not volatile temporary var is UB. Loading can be reordered.</t>
-  </si>
-  <si>
-    <t>hard to categorize</t>
-  </si>
-  <si>
-    <t>bc1fb82ae11753c5dec53c667a055dc37796dbd2</t>
-  </si>
-  <si>
-    <t>preventive</t>
   </si>
   <si>
     <t>UB dma data race</t>
@@ -1216,10 +1093,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>new</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>1(linux)</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -1349,16 +1222,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>a9a3ed1eff3601b63aea4fb462d8b3b92c7c1e7e</t>
-  </si>
-  <si>
-    <t>register spill</t>
-    <phoneticPr fontId="22" type="noConversion"/>
-  </si>
-  <si>
-    <t>2c88c742d011707b55da7b54b06a030c6f57233f</t>
-  </si>
-  <si>
     <t>3(gcc)</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -1422,15 +1285,59 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>tail call optimization</t>
-    <phoneticPr fontId="22" type="noConversion"/>
-  </si>
-  <si>
     <t>DB type demotion</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>Default Behavior</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>b-27</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>b-28</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>b-29</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>b-30</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-50</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-51</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-52</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-53</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>b-31</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-54</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-55</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>l-56</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -2450,7 +2357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59979BBC-FF03-4FA8-9496-87716FB7753F}">
-  <dimension ref="A1:M236"/>
+  <dimension ref="A1:M231"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" customWidth="1"/>
@@ -2615,7 +2522,7 @@
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>399</v>
+        <v>357</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -2644,7 +2551,7 @@
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
@@ -2667,19 +2574,19 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>297</v>
+        <v>256</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>241</v>
+        <v>200</v>
       </c>
       <c r="C8" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D8" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>298</v>
+        <v>257</v>
       </c>
       <c r="F8" s="7">
         <v>2024</v>
@@ -2688,10 +2595,10 @@
         <v>2006</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -2702,7 +2609,7 @@
         <v>27</v>
       </c>
       <c r="C9" t="s">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -2731,7 +2638,7 @@
         <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
@@ -2754,16 +2661,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>240</v>
+        <v>199</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>241</v>
+        <v>200</v>
       </c>
       <c r="C11" t="s">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="D11" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E11">
         <v>115770</v>
@@ -2775,10 +2682,10 @@
         <v>2006</v>
       </c>
       <c r="H11" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I11" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -2812,16 +2719,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>242</v>
+        <v>201</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>356</v>
+        <v>315</v>
       </c>
       <c r="D13" t="s">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="E13">
         <v>122400</v>
@@ -2833,24 +2740,24 @@
         <v>2007</v>
       </c>
       <c r="H13" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I13" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>242</v>
+        <v>201</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>356</v>
+        <v>315</v>
       </c>
       <c r="D14" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E14">
         <v>106333</v>
@@ -2862,10 +2769,10 @@
         <v>2007</v>
       </c>
       <c r="H14" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I14" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -2876,13 +2783,13 @@
         <v>35</v>
       </c>
       <c r="C15" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D15" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>302</v>
+        <v>261</v>
       </c>
       <c r="F15" s="3">
         <v>2013</v>
@@ -2891,10 +2798,10 @@
         <v>2007</v>
       </c>
       <c r="H15" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -2905,13 +2812,13 @@
         <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D16" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>303</v>
+        <v>262</v>
       </c>
       <c r="F16" s="3">
         <v>2012</v>
@@ -2920,10 +2827,10 @@
         <v>2007</v>
       </c>
       <c r="H16" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
@@ -2934,13 +2841,13 @@
         <v>35</v>
       </c>
       <c r="C17" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D17" t="s">
         <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>406</v>
+        <v>361</v>
       </c>
       <c r="F17">
         <v>2013</v>
@@ -2972,13 +2879,13 @@
         <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D18" t="s">
         <v>36</v>
       </c>
       <c r="E18" t="s">
-        <v>407</v>
+        <v>362</v>
       </c>
       <c r="F18">
         <v>2015</v>
@@ -3010,7 +2917,7 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
@@ -3039,13 +2946,13 @@
         <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D20" t="s">
         <v>36</v>
       </c>
       <c r="E20" t="s">
-        <v>408</v>
+        <v>363</v>
       </c>
       <c r="F20">
         <v>2017</v>
@@ -3077,7 +2984,7 @@
         <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D21" t="s">
         <v>22</v>
@@ -3106,7 +3013,7 @@
         <v>35</v>
       </c>
       <c r="C22" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D22" t="s">
         <v>22</v>
@@ -3135,13 +3042,13 @@
         <v>35</v>
       </c>
       <c r="C23" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D23" t="s">
         <v>36</v>
       </c>
       <c r="E23" t="s">
-        <v>409</v>
+        <v>364</v>
       </c>
       <c r="F23">
         <v>2020</v>
@@ -3173,7 +3080,7 @@
         <v>35</v>
       </c>
       <c r="C24" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
@@ -3202,7 +3109,7 @@
         <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D25" t="s">
         <v>22</v>
@@ -3231,7 +3138,7 @@
         <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D26" t="s">
         <v>22</v>
@@ -3260,7 +3167,7 @@
         <v>35</v>
       </c>
       <c r="C27" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D27" t="s">
         <v>22</v>
@@ -3289,7 +3196,7 @@
         <v>35</v>
       </c>
       <c r="C28" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D28" t="s">
         <v>22</v>
@@ -3318,7 +3225,7 @@
         <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D29" t="s">
         <v>22</v>
@@ -3347,7 +3254,7 @@
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D30" t="s">
         <v>22</v>
@@ -3376,7 +3283,7 @@
         <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -3405,7 +3312,7 @@
         <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -3434,7 +3341,7 @@
         <v>35</v>
       </c>
       <c r="C33" t="s">
-        <v>355</v>
+        <v>314</v>
       </c>
       <c r="D33" t="s">
         <v>22</v>
@@ -3457,16 +3364,16 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>244</v>
+        <v>203</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C34" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D34" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E34">
         <v>115019</v>
@@ -3478,24 +3385,24 @@
         <v>2007</v>
       </c>
       <c r="H34" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I34" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>244</v>
+        <v>203</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D35" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E35">
         <v>114554</v>
@@ -3507,24 +3414,24 @@
         <v>2007</v>
       </c>
       <c r="H35" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I35" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>244</v>
+        <v>203</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C36" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D36" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E36">
         <v>107785</v>
@@ -3536,10 +3443,10 @@
         <v>2007</v>
       </c>
       <c r="H36" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I36" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
@@ -3550,7 +3457,7 @@
         <v>35</v>
       </c>
       <c r="C37" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D37" t="s">
         <v>22</v>
@@ -3579,7 +3486,7 @@
         <v>35</v>
       </c>
       <c r="C38" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D38" t="s">
         <v>22</v>
@@ -3608,7 +3515,7 @@
         <v>35</v>
       </c>
       <c r="C39" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D39" t="s">
         <v>22</v>
@@ -3637,7 +3544,7 @@
         <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D40" t="s">
         <v>22</v>
@@ -3666,7 +3573,7 @@
         <v>35</v>
       </c>
       <c r="C41" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D41" t="s">
         <v>22</v>
@@ -3695,7 +3602,7 @@
         <v>35</v>
       </c>
       <c r="C42" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D42" t="s">
         <v>22</v>
@@ -3724,13 +3631,13 @@
         <v>35</v>
       </c>
       <c r="C43" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D43" t="s">
         <v>36</v>
       </c>
       <c r="E43" t="s">
-        <v>411</v>
+        <v>366</v>
       </c>
       <c r="F43">
         <v>2012</v>
@@ -3762,13 +3669,13 @@
         <v>35</v>
       </c>
       <c r="C44" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D44" t="s">
         <v>36</v>
       </c>
       <c r="E44" t="s">
-        <v>412</v>
+        <v>367</v>
       </c>
       <c r="F44">
         <v>2011</v>
@@ -3800,7 +3707,7 @@
         <v>35</v>
       </c>
       <c r="C45" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D45" t="s">
         <v>22</v>
@@ -3829,7 +3736,7 @@
         <v>35</v>
       </c>
       <c r="C46" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D46" t="s">
         <v>22</v>
@@ -3858,7 +3765,7 @@
         <v>35</v>
       </c>
       <c r="C47" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D47" t="s">
         <v>22</v>
@@ -3887,7 +3794,7 @@
         <v>35</v>
       </c>
       <c r="C48" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D48" t="s">
         <v>22</v>
@@ -3916,7 +3823,7 @@
         <v>35</v>
       </c>
       <c r="C49" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -3945,7 +3852,7 @@
         <v>35</v>
       </c>
       <c r="C50" t="s">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="D50" t="s">
         <v>22</v>
@@ -4067,7 +3974,7 @@
         <v>36</v>
       </c>
       <c r="E54" t="s">
-        <v>413</v>
+        <v>368</v>
       </c>
       <c r="F54">
         <v>2013</v>
@@ -4105,7 +4012,7 @@
         <v>36</v>
       </c>
       <c r="E55" t="s">
-        <v>414</v>
+        <v>369</v>
       </c>
       <c r="F55">
         <v>2013</v>
@@ -4189,13 +4096,13 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>227</v>
+        <v>186</v>
       </c>
       <c r="B58" t="s">
         <v>52</v>
       </c>
       <c r="C58" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -4218,19 +4125,19 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>254</v>
+        <v>213</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>255</v>
+        <v>214</v>
       </c>
       <c r="C59" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D59" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>256</v>
+        <v>215</v>
       </c>
       <c r="F59">
         <v>2020</v>
@@ -4247,13 +4154,13 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>226</v>
+        <v>185</v>
       </c>
       <c r="B60" t="s">
         <v>52</v>
       </c>
       <c r="C60" t="s">
-        <v>404</v>
+        <v>359</v>
       </c>
       <c r="D60" t="s">
         <v>22</v>
@@ -4276,19 +4183,19 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>237</v>
+        <v>196</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C61" t="s">
-        <v>404</v>
+        <v>359</v>
       </c>
       <c r="D61" t="s">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="E61" t="s">
-        <v>238</v>
+        <v>197</v>
       </c>
       <c r="F61">
         <v>2019</v>
@@ -4297,10 +4204,10 @@
         <v>2009</v>
       </c>
       <c r="H61" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I61" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
@@ -4308,10 +4215,10 @@
         <v>54</v>
       </c>
       <c r="B62" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>337</v>
+        <v>296</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>22</v>
@@ -4338,10 +4245,10 @@
         <v>54</v>
       </c>
       <c r="B63" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>337</v>
+        <v>296</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>22</v>
@@ -4365,16 +4272,16 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
-        <v>334</v>
+        <v>293</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>336</v>
+        <v>295</v>
       </c>
       <c r="D64" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E64" s="8">
         <v>86947</v>
@@ -4395,16 +4302,16 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
-        <v>334</v>
+        <v>293</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>336</v>
+        <v>295</v>
       </c>
       <c r="D65" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E65">
         <v>110530</v>
@@ -4425,16 +4332,16 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
-        <v>334</v>
+        <v>293</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>336</v>
+        <v>295</v>
       </c>
       <c r="D66" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E66">
         <v>112409</v>
@@ -4455,19 +4362,19 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
-        <v>334</v>
+        <v>293</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>336</v>
+        <v>295</v>
       </c>
       <c r="D67" t="s">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="E67" t="s">
-        <v>335</v>
+        <v>294</v>
       </c>
       <c r="F67">
         <v>2015</v>
@@ -4476,25 +4383,25 @@
         <v>2009</v>
       </c>
       <c r="H67" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I67" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
       <c r="J67" s="2"/>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
-        <v>334</v>
+        <v>293</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>333</v>
+        <v>292</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>336</v>
+        <v>295</v>
       </c>
       <c r="D68" t="s">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="E68">
         <v>78154</v>
@@ -4506,10 +4413,10 @@
         <v>2009</v>
       </c>
       <c r="H68" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I68" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
       <c r="J68" s="2"/>
     </row>
@@ -4518,7 +4425,7 @@
         <v>55</v>
       </c>
       <c r="B69" t="s">
-        <v>222</v>
+        <v>181</v>
       </c>
       <c r="C69" t="s">
         <v>21</v>
@@ -4544,19 +4451,19 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>330</v>
+        <v>289</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>331</v>
+        <v>290</v>
       </c>
       <c r="C70" t="s">
-        <v>357</v>
+        <v>316</v>
       </c>
       <c r="D70" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>332</v>
+        <v>291</v>
       </c>
       <c r="F70" s="3">
         <v>2016</v>
@@ -4565,10 +4472,10 @@
         <v>2015</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.2">
@@ -4579,7 +4486,7 @@
         <v>57</v>
       </c>
       <c r="C71" t="s">
-        <v>357</v>
+        <v>316</v>
       </c>
       <c r="D71" t="s">
         <v>22</v>
@@ -4608,13 +4515,13 @@
         <v>57</v>
       </c>
       <c r="C72" t="s">
-        <v>357</v>
+        <v>316</v>
       </c>
       <c r="D72" t="s">
         <v>36</v>
       </c>
       <c r="E72" t="s">
-        <v>415</v>
+        <v>370</v>
       </c>
       <c r="F72">
         <v>2021</v>
@@ -4640,16 +4547,16 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
-        <v>246</v>
+        <v>205</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>60</v>
       </c>
       <c r="C73" t="s">
-        <v>354</v>
+        <v>313</v>
       </c>
       <c r="D73" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E73">
         <v>29967</v>
@@ -4669,16 +4576,16 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>246</v>
+        <v>205</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>60</v>
       </c>
       <c r="C74" t="s">
-        <v>354</v>
+        <v>313</v>
       </c>
       <c r="D74" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E74">
         <v>18723</v>
@@ -4704,10 +4611,10 @@
         <v>60</v>
       </c>
       <c r="C75" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D75" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E75">
         <v>112442</v>
@@ -4727,19 +4634,19 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
-        <v>246</v>
+        <v>205</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>304</v>
+        <v>263</v>
       </c>
       <c r="C76" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D76" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>198</v>
+        <v>179</v>
       </c>
       <c r="F76" s="3">
         <v>2024</v>
@@ -4748,10 +4655,10 @@
         <v>2024</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.2">
@@ -4762,7 +4669,7 @@
         <v>60</v>
       </c>
       <c r="C77" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D77" t="s">
         <v>22</v>
@@ -4791,7 +4698,7 @@
         <v>60</v>
       </c>
       <c r="C78" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D78" t="s">
         <v>22</v>
@@ -4820,7 +4727,7 @@
         <v>60</v>
       </c>
       <c r="C79" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D79" t="s">
         <v>22</v>
@@ -4849,7 +4756,7 @@
         <v>60</v>
       </c>
       <c r="C80" t="s">
-        <v>341</v>
+        <v>300</v>
       </c>
       <c r="D80" t="s">
         <v>22</v>
@@ -4872,19 +4779,19 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
-        <v>314</v>
+        <v>273</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>315</v>
+        <v>274</v>
       </c>
       <c r="C81" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D81" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="F81" s="3">
         <v>2024</v>
@@ -4893,27 +4800,27 @@
         <v>2008</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>314</v>
+        <v>273</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>315</v>
+        <v>274</v>
       </c>
       <c r="C82" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D82" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>316</v>
+        <v>275</v>
       </c>
       <c r="F82" s="3">
         <v>2015</v>
@@ -4922,27 +4829,27 @@
         <v>2008</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>314</v>
+        <v>273</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>315</v>
+        <v>274</v>
       </c>
       <c r="C83" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D83" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>317</v>
+        <v>276</v>
       </c>
       <c r="F83" s="3">
         <v>2008</v>
@@ -4951,10 +4858,10 @@
         <v>2008</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.2">
@@ -4965,7 +4872,7 @@
         <v>62</v>
       </c>
       <c r="C84" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D84" t="s">
         <v>12</v>
@@ -5017,16 +4924,16 @@
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
-        <v>247</v>
+        <v>206</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C86" t="s">
-        <v>344</v>
+        <v>303</v>
       </c>
       <c r="D86" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E86">
         <v>27299</v>
@@ -5038,10 +4945,10 @@
         <v>2006</v>
       </c>
       <c r="H86" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I86" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.2">
@@ -5052,13 +4959,13 @@
         <v>68</v>
       </c>
       <c r="C87" t="s">
-        <v>344</v>
+        <v>303</v>
       </c>
       <c r="D87" t="s">
         <v>36</v>
       </c>
       <c r="E87" t="s">
-        <v>416</v>
+        <v>371</v>
       </c>
       <c r="F87">
         <v>2017</v>
@@ -5090,7 +4997,7 @@
         <v>68</v>
       </c>
       <c r="C88" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="D88" t="s">
         <v>22</v>
@@ -5119,7 +5026,7 @@
         <v>68</v>
       </c>
       <c r="C89" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="D89" t="s">
         <v>22</v>
@@ -5148,7 +5055,7 @@
         <v>68</v>
       </c>
       <c r="C90" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="D90" t="s">
         <v>22</v>
@@ -5177,7 +5084,7 @@
         <v>68</v>
       </c>
       <c r="C91" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="D91" t="s">
         <v>22</v>
@@ -5200,16 +5107,16 @@
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>385</v>
+        <v>343</v>
       </c>
       <c r="C92" t="s">
-        <v>367</v>
+        <v>325</v>
       </c>
       <c r="D92" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E92">
         <v>43774</v>
@@ -5221,10 +5128,10 @@
         <v>2010</v>
       </c>
       <c r="H92" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I92" t="s">
-        <v>386</v>
+        <v>344</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.2">
@@ -5235,7 +5142,7 @@
         <v>70</v>
       </c>
       <c r="C93" t="s">
-        <v>340</v>
+        <v>299</v>
       </c>
       <c r="D93" t="s">
         <v>12</v>
@@ -5258,16 +5165,16 @@
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
-        <v>248</v>
+        <v>207</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C94" t="s">
-        <v>340</v>
+        <v>299</v>
       </c>
       <c r="D94" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E94">
         <v>60918</v>
@@ -5293,10 +5200,10 @@
         <v>70</v>
       </c>
       <c r="C95" t="s">
-        <v>339</v>
+        <v>298</v>
       </c>
       <c r="D95" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E95">
         <v>52492</v>
@@ -5322,10 +5229,10 @@
         <v>70</v>
       </c>
       <c r="C96" t="s">
-        <v>339</v>
+        <v>298</v>
       </c>
       <c r="D96" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E96">
         <v>22447</v>
@@ -5351,10 +5258,10 @@
         <v>70</v>
       </c>
       <c r="C97" t="s">
-        <v>339</v>
+        <v>298</v>
       </c>
       <c r="D97" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E97">
         <v>116856</v>
@@ -5380,10 +5287,10 @@
         <v>70</v>
       </c>
       <c r="C98" t="s">
-        <v>339</v>
+        <v>298</v>
       </c>
       <c r="D98" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E98">
         <v>114080</v>
@@ -5467,13 +5374,13 @@
         <v>76</v>
       </c>
       <c r="C101" t="s">
-        <v>342</v>
+        <v>301</v>
       </c>
       <c r="D101" t="s">
         <v>36</v>
       </c>
       <c r="E101" t="s">
-        <v>417</v>
+        <v>372</v>
       </c>
       <c r="F101">
         <v>2011</v>
@@ -5505,7 +5412,7 @@
         <v>76</v>
       </c>
       <c r="C102" t="s">
-        <v>342</v>
+        <v>301</v>
       </c>
       <c r="D102" t="s">
         <v>22</v>
@@ -5528,16 +5435,16 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
-        <v>249</v>
+        <v>208</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>250</v>
+        <v>209</v>
       </c>
       <c r="C103" t="s">
-        <v>342</v>
+        <v>301</v>
       </c>
       <c r="D103" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E103">
         <v>29094</v>
@@ -5549,27 +5456,27 @@
         <v>2006</v>
       </c>
       <c r="H103" t="s">
-        <v>251</v>
+        <v>210</v>
       </c>
       <c r="I103" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
-        <v>249</v>
+        <v>208</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>250</v>
+        <v>209</v>
       </c>
       <c r="C104" t="s">
-        <v>342</v>
+        <v>301</v>
       </c>
       <c r="D104" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>253</v>
+        <v>212</v>
       </c>
       <c r="F104">
         <v>2022</v>
@@ -5578,10 +5485,10 @@
         <v>2006</v>
       </c>
       <c r="H104" t="s">
-        <v>251</v>
+        <v>210</v>
       </c>
       <c r="I104" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.2">
@@ -5592,7 +5499,7 @@
         <v>79</v>
       </c>
       <c r="C105" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D105" t="s">
         <v>12</v>
@@ -5615,19 +5522,19 @@
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
-        <v>299</v>
+        <v>258</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>300</v>
+        <v>259</v>
       </c>
       <c r="C106" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D106" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>318</v>
+        <v>277</v>
       </c>
       <c r="F106" s="3">
         <v>2020</v>
@@ -5636,27 +5543,27 @@
         <v>2017</v>
       </c>
       <c r="H106" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>299</v>
+        <v>258</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>300</v>
+        <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D107" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>301</v>
+        <v>260</v>
       </c>
       <c r="F107" s="3">
         <v>2017</v>
@@ -5665,10 +5572,10 @@
         <v>2017</v>
       </c>
       <c r="H107" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.2">
@@ -5676,7 +5583,7 @@
         <v>81</v>
       </c>
       <c r="B108" t="s">
-        <v>223</v>
+        <v>182</v>
       </c>
       <c r="C108" t="s">
         <v>83</v>
@@ -5731,16 +5638,16 @@
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>370</v>
+        <v>328</v>
       </c>
       <c r="C110" t="s">
-        <v>367</v>
+        <v>325</v>
       </c>
       <c r="D110" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E110">
         <v>48623</v>
@@ -5752,24 +5659,24 @@
         <v>2011</v>
       </c>
       <c r="H110" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I110" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
-        <v>365</v>
+        <v>378</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>371</v>
+        <v>329</v>
       </c>
       <c r="C111" t="s">
-        <v>372</v>
+        <v>330</v>
       </c>
       <c r="D111" t="s">
-        <v>373</v>
+        <v>331</v>
       </c>
       <c r="E111" s="3">
         <v>61112</v>
@@ -5781,24 +5688,24 @@
         <v>2023</v>
       </c>
       <c r="H111" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I111" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
-        <v>365</v>
+        <v>379</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>382</v>
+        <v>340</v>
       </c>
       <c r="C112" t="s">
-        <v>367</v>
+        <v>325</v>
       </c>
       <c r="D112" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E112" s="3">
         <v>106635</v>
@@ -5810,10 +5717,10 @@
         <v>2022</v>
       </c>
       <c r="H112" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I112" t="s">
-        <v>239</v>
+        <v>198</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.2">
@@ -5853,7 +5760,7 @@
         <v>91</v>
       </c>
       <c r="C114" t="s">
-        <v>347</v>
+        <v>306</v>
       </c>
       <c r="D114" t="s">
         <v>12</v>
@@ -5882,13 +5789,13 @@
         <v>91</v>
       </c>
       <c r="C115" t="s">
-        <v>347</v>
+        <v>306</v>
       </c>
       <c r="D115" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>320</v>
+        <v>279</v>
       </c>
       <c r="F115" s="3">
         <v>2023</v>
@@ -5897,7 +5804,7 @@
         <v>2005</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I115" t="s">
         <v>89</v>
@@ -5911,13 +5818,13 @@
         <v>91</v>
       </c>
       <c r="C116" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D116" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>321</v>
+        <v>280</v>
       </c>
       <c r="F116" s="3">
         <v>2023</v>
@@ -5926,7 +5833,7 @@
         <v>2005</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I116" t="s">
         <v>89</v>
@@ -5940,13 +5847,13 @@
         <v>91</v>
       </c>
       <c r="C117" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D117" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>322</v>
+        <v>281</v>
       </c>
       <c r="F117" s="3">
         <v>2023</v>
@@ -5955,7 +5862,7 @@
         <v>2005</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I117" t="s">
         <v>89</v>
@@ -5969,13 +5876,13 @@
         <v>91</v>
       </c>
       <c r="C118" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D118" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>323</v>
+        <v>282</v>
       </c>
       <c r="F118" s="3">
         <v>2023</v>
@@ -5984,7 +5891,7 @@
         <v>2005</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I118" t="s">
         <v>89</v>
@@ -5998,13 +5905,13 @@
         <v>91</v>
       </c>
       <c r="C119" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D119" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>324</v>
+        <v>283</v>
       </c>
       <c r="F119" s="3">
         <v>2012</v>
@@ -6013,7 +5920,7 @@
         <v>2005</v>
       </c>
       <c r="H119" s="3" t="s">
-        <v>319</v>
+        <v>278</v>
       </c>
       <c r="I119" t="s">
         <v>89</v>
@@ -6021,16 +5928,16 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
-        <v>229</v>
+        <v>188</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C120" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D120" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E120">
         <v>67246</v>
@@ -6042,24 +5949,24 @@
         <v>2005</v>
       </c>
       <c r="H120" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I120" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
-        <v>229</v>
+        <v>188</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C121" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D121" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E121">
         <v>57862</v>
@@ -6071,7 +5978,7 @@
         <v>2005</v>
       </c>
       <c r="H121" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I121" t="s">
         <v>89</v>
@@ -6085,10 +5992,10 @@
         <v>91</v>
       </c>
       <c r="C122" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D122" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E122">
         <v>45819</v>
@@ -6100,7 +6007,7 @@
         <v>2005</v>
       </c>
       <c r="H122" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I122" t="s">
         <v>89</v>
@@ -6114,10 +6021,10 @@
         <v>91</v>
       </c>
       <c r="C123" t="s">
-        <v>346</v>
+        <v>305</v>
       </c>
       <c r="D123" t="s">
-        <v>230</v>
+        <v>189</v>
       </c>
       <c r="E123">
         <v>21387</v>
@@ -6129,7 +6036,7 @@
         <v>2005</v>
       </c>
       <c r="H123" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I123" t="s">
         <v>89</v>
@@ -6143,7 +6050,7 @@
         <v>94</v>
       </c>
       <c r="C124" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D124" t="s">
         <v>12</v>
@@ -6166,19 +6073,19 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" s="5" t="s">
-        <v>261</v>
+        <v>220</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>262</v>
+        <v>221</v>
       </c>
       <c r="C125" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D125" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>263</v>
+        <v>222</v>
       </c>
       <c r="F125">
         <v>2021</v>
@@ -6187,27 +6094,27 @@
         <v>2006</v>
       </c>
       <c r="H125" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I125" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A126" s="5" t="s">
-        <v>261</v>
+        <v>220</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>262</v>
+        <v>221</v>
       </c>
       <c r="C126" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D126" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>328</v>
+        <v>287</v>
       </c>
       <c r="F126" s="3">
         <v>2011</v>
@@ -6216,27 +6123,27 @@
         <v>2006</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I126" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" s="5" t="s">
-        <v>261</v>
+        <v>220</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>262</v>
+        <v>221</v>
       </c>
       <c r="C127" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D127" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>329</v>
+        <v>288</v>
       </c>
       <c r="F127" s="3">
         <v>2006</v>
@@ -6245,10 +6152,10 @@
         <v>2006</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I127" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.2">
@@ -6282,19 +6189,19 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>388</v>
+        <v>346</v>
       </c>
       <c r="C129" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D129" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>387</v>
+        <v>345</v>
       </c>
       <c r="F129">
         <v>2023</v>
@@ -6303,27 +6210,27 @@
         <v>2023</v>
       </c>
       <c r="H129" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I129" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" s="5" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>420</v>
+        <v>374</v>
       </c>
       <c r="C130" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D130" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>390</v>
+        <v>348</v>
       </c>
       <c r="F130">
         <v>2021</v>
@@ -6332,10 +6239,10 @@
         <v>2021</v>
       </c>
       <c r="H130" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I130" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.2">
@@ -6398,19 +6305,19 @@
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
-        <v>365</v>
+        <v>382</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>377</v>
+        <v>335</v>
       </c>
       <c r="C133" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D133" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>378</v>
+        <v>336</v>
       </c>
       <c r="F133">
         <v>2022</v>
@@ -6419,10 +6326,10 @@
         <v>2022</v>
       </c>
       <c r="H133" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I133" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.2">
@@ -6430,7 +6337,7 @@
         <v>101</v>
       </c>
       <c r="B134" t="s">
-        <v>228</v>
+        <v>187</v>
       </c>
       <c r="C134" t="s">
         <v>11</v>
@@ -6456,19 +6363,19 @@
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>380</v>
+        <v>338</v>
       </c>
       <c r="C135" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D135" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>381</v>
+        <v>339</v>
       </c>
       <c r="F135">
         <v>2021</v>
@@ -6477,24 +6384,24 @@
         <v>2021</v>
       </c>
       <c r="H135" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I135" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>395</v>
+        <v>353</v>
       </c>
       <c r="C136" t="s">
-        <v>396</v>
+        <v>354</v>
       </c>
       <c r="D136" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E136" s="3">
         <v>50314</v>
@@ -6506,24 +6413,24 @@
         <v>2008</v>
       </c>
       <c r="H136" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I136" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>395</v>
+        <v>353</v>
       </c>
       <c r="C137" t="s">
-        <v>396</v>
+        <v>354</v>
       </c>
       <c r="D137" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E137" s="3">
         <v>34736</v>
@@ -6535,10 +6442,10 @@
         <v>2008</v>
       </c>
       <c r="H137" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I137" t="s">
-        <v>379</v>
+        <v>337</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.2">
@@ -6549,13 +6456,13 @@
         <v>104</v>
       </c>
       <c r="C138" t="s">
-        <v>349</v>
+        <v>308</v>
       </c>
       <c r="D138" t="s">
         <v>12</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>225</v>
+        <v>184</v>
       </c>
       <c r="F138">
         <v>2023</v>
@@ -6572,19 +6479,19 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
-        <v>276</v>
+        <v>235</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C139" t="s">
-        <v>349</v>
+        <v>308</v>
       </c>
       <c r="D139" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>278</v>
+        <v>237</v>
       </c>
       <c r="F139" s="3">
         <v>2015</v>
@@ -6593,10 +6500,10 @@
         <v>2005</v>
       </c>
       <c r="H139" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I139" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.2">
@@ -6607,13 +6514,13 @@
         <v>104</v>
       </c>
       <c r="C140" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D140" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>279</v>
+        <v>238</v>
       </c>
       <c r="F140" s="3">
         <v>2011</v>
@@ -6622,10 +6529,10 @@
         <v>2005</v>
       </c>
       <c r="H140" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I140" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.2">
@@ -6633,16 +6540,16 @@
         <v>103</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C141" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D141" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>280</v>
+        <v>239</v>
       </c>
       <c r="F141" s="3">
         <v>2005</v>
@@ -6651,10 +6558,10 @@
         <v>2005</v>
       </c>
       <c r="H141" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I141" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.2">
@@ -6665,13 +6572,13 @@
         <v>104</v>
       </c>
       <c r="C142" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D142" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>281</v>
+        <v>240</v>
       </c>
       <c r="F142" s="3">
         <v>2025</v>
@@ -6680,10 +6587,10 @@
         <v>2005</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I142" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.2">
@@ -6691,16 +6598,16 @@
         <v>103</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C143" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D143" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>283</v>
+        <v>242</v>
       </c>
       <c r="F143" s="3">
         <v>2025</v>
@@ -6709,10 +6616,10 @@
         <v>2005</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I143" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.2">
@@ -6723,13 +6630,13 @@
         <v>104</v>
       </c>
       <c r="C144" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D144" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>285</v>
+        <v>244</v>
       </c>
       <c r="F144" s="3">
         <v>2024</v>
@@ -6738,10 +6645,10 @@
         <v>2005</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I144" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.2">
@@ -6749,16 +6656,16 @@
         <v>103</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C145" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D145" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>286</v>
+        <v>245</v>
       </c>
       <c r="F145" s="3">
         <v>2023</v>
@@ -6767,10 +6674,10 @@
         <v>2005</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I145" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.2">
@@ -6781,13 +6688,13 @@
         <v>104</v>
       </c>
       <c r="C146" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D146" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>287</v>
+        <v>246</v>
       </c>
       <c r="F146" s="3">
         <v>2021</v>
@@ -6796,10 +6703,10 @@
         <v>2005</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I146" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.2">
@@ -6807,16 +6714,16 @@
         <v>103</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C147" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D147" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>288</v>
+        <v>247</v>
       </c>
       <c r="F147" s="3">
         <v>2018</v>
@@ -6825,10 +6732,10 @@
         <v>2005</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I147" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.2">
@@ -6839,13 +6746,13 @@
         <v>104</v>
       </c>
       <c r="C148" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D148" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>289</v>
+        <v>248</v>
       </c>
       <c r="F148" s="3">
         <v>2012</v>
@@ -6854,10 +6761,10 @@
         <v>2005</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I148" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.2">
@@ -6865,16 +6772,16 @@
         <v>103</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>277</v>
+        <v>236</v>
       </c>
       <c r="C149" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D149" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E149" s="3" t="s">
-        <v>290</v>
+        <v>249</v>
       </c>
       <c r="F149" s="3">
         <v>2012</v>
@@ -6883,10 +6790,10 @@
         <v>2005</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I149" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.2">
@@ -6897,13 +6804,13 @@
         <v>104</v>
       </c>
       <c r="C150" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D150" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E150" s="3" t="s">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="F150" s="3">
         <v>2007</v>
@@ -6912,10 +6819,10 @@
         <v>2005</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I150" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.2">
@@ -6926,13 +6833,13 @@
         <v>104</v>
       </c>
       <c r="C151" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D151" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E151" s="3" t="s">
-        <v>292</v>
+        <v>251</v>
       </c>
       <c r="F151" s="3">
         <v>2006</v>
@@ -6941,10 +6848,10 @@
         <v>2005</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>284</v>
+        <v>243</v>
       </c>
       <c r="I151" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.2">
@@ -6955,13 +6862,13 @@
         <v>104</v>
       </c>
       <c r="C152" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D152" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E152" s="3" t="s">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="F152" s="3">
         <v>2024</v>
@@ -6970,10 +6877,10 @@
         <v>2005</v>
       </c>
       <c r="H152" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I152" s="3" t="s">
-        <v>232</v>
+        <v>191</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.2">
@@ -6981,7 +6888,7 @@
         <v>105</v>
       </c>
       <c r="B153" t="s">
-        <v>358</v>
+        <v>317</v>
       </c>
       <c r="C153" t="s">
         <v>21</v>
@@ -7010,7 +6917,7 @@
         <v>107</v>
       </c>
       <c r="B154" t="s">
-        <v>359</v>
+        <v>318</v>
       </c>
       <c r="C154" t="s">
         <v>11</v>
@@ -7036,19 +6943,19 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A155" s="5" t="s">
-        <v>365</v>
+        <v>385</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>383</v>
+        <v>341</v>
       </c>
       <c r="C155" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D155" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E155" s="3" t="s">
-        <v>384</v>
+        <v>342</v>
       </c>
       <c r="F155" s="3">
         <v>2023</v>
@@ -7057,10 +6964,10 @@
         <v>2023</v>
       </c>
       <c r="H155" s="3" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I155" t="s">
-        <v>363</v>
+        <v>322</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.2">
@@ -7071,7 +6978,7 @@
         <v>110</v>
       </c>
       <c r="C156" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D156" t="s">
         <v>12</v>
@@ -7094,19 +7001,19 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
-        <v>325</v>
+        <v>284</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>326</v>
+        <v>285</v>
       </c>
       <c r="C157" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D157" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E157" s="3" t="s">
-        <v>327</v>
+        <v>286</v>
       </c>
       <c r="F157" s="3">
         <v>2011</v>
@@ -7115,10 +7022,10 @@
         <v>2011</v>
       </c>
       <c r="H157" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I157" s="3" t="s">
-        <v>260</v>
+        <v>219</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.2">
@@ -7126,7 +7033,7 @@
         <v>112</v>
       </c>
       <c r="B158" t="s">
-        <v>374</v>
+        <v>332</v>
       </c>
       <c r="C158" t="s">
         <v>11</v>
@@ -7152,19 +7059,19 @@
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
-        <v>360</v>
+        <v>319</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>389</v>
+        <v>347</v>
       </c>
       <c r="C159" t="s">
-        <v>364</v>
+        <v>323</v>
       </c>
       <c r="D159" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E159" s="3" t="s">
-        <v>362</v>
+        <v>321</v>
       </c>
       <c r="F159">
         <v>2018</v>
@@ -7173,10 +7080,10 @@
         <v>2008</v>
       </c>
       <c r="H159" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I159" t="s">
-        <v>363</v>
+        <v>322</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.2">
@@ -7184,10 +7091,10 @@
         <v>114</v>
       </c>
       <c r="B160" t="s">
-        <v>389</v>
+        <v>347</v>
       </c>
       <c r="C160" t="s">
-        <v>364</v>
+        <v>323</v>
       </c>
       <c r="D160" t="s">
         <v>12</v>
@@ -7239,19 +7146,19 @@
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A162" s="4" t="s">
-        <v>365</v>
+        <v>386</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>375</v>
+        <v>333</v>
       </c>
       <c r="C162" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D162" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E162" s="3" t="s">
-        <v>376</v>
+        <v>334</v>
       </c>
       <c r="F162">
         <v>2022</v>
@@ -7260,10 +7167,10 @@
         <v>2022</v>
       </c>
       <c r="H162" t="s">
-        <v>369</v>
+        <v>327</v>
       </c>
       <c r="I162" t="s">
-        <v>363</v>
+        <v>322</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.2">
@@ -7271,16 +7178,16 @@
         <v>119</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>313</v>
+        <v>272</v>
       </c>
       <c r="C163" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D163" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E163" s="3" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="F163" s="3">
         <v>2023</v>
@@ -7303,13 +7210,13 @@
         <v>120</v>
       </c>
       <c r="C164" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D164" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E164" s="3" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="F164" s="3">
         <v>2023</v>
@@ -7326,19 +7233,19 @@
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
-        <v>312</v>
+        <v>271</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>313</v>
+        <v>272</v>
       </c>
       <c r="C165" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D165" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E165" s="3" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
       <c r="F165" s="3">
         <v>2024</v>
@@ -7361,7 +7268,7 @@
         <v>120</v>
       </c>
       <c r="C166" t="s">
-        <v>338</v>
+        <v>297</v>
       </c>
       <c r="D166" t="s">
         <v>12</v>
@@ -7413,19 +7320,19 @@
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A168" s="4" t="s">
-        <v>310</v>
+        <v>269</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>311</v>
+        <v>270</v>
       </c>
       <c r="C168" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D168" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E168" s="3" t="s">
-        <v>308</v>
+        <v>267</v>
       </c>
       <c r="F168" s="3">
         <v>2012</v>
@@ -7434,7 +7341,7 @@
         <v>2012</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I168" t="s">
         <v>106</v>
@@ -7442,19 +7349,19 @@
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A169" s="5" t="s">
-        <v>310</v>
+        <v>269</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>311</v>
+        <v>270</v>
       </c>
       <c r="C169" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D169" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E169" s="3" t="s">
-        <v>309</v>
+        <v>268</v>
       </c>
       <c r="F169" s="3">
         <v>2012</v>
@@ -7463,7 +7370,7 @@
         <v>2012</v>
       </c>
       <c r="H169" s="3" t="s">
-        <v>282</v>
+        <v>241</v>
       </c>
       <c r="I169" t="s">
         <v>106</v>
@@ -7477,7 +7384,7 @@
         <v>127</v>
       </c>
       <c r="C170" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D170" t="s">
         <v>12</v>
@@ -7506,7 +7413,7 @@
         <v>130</v>
       </c>
       <c r="C171" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D171" t="s">
         <v>12</v>
@@ -7535,7 +7442,7 @@
         <v>130</v>
       </c>
       <c r="C172" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D172" t="s">
         <v>12</v>
@@ -7558,19 +7465,19 @@
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A173" s="4" t="s">
-        <v>257</v>
+        <v>216</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>258</v>
+        <v>217</v>
       </c>
       <c r="C173" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D173" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>259</v>
+        <v>218</v>
       </c>
       <c r="F173">
         <v>2015</v>
@@ -7579,10 +7486,10 @@
         <v>2006</v>
       </c>
       <c r="H173" t="s">
-        <v>245</v>
+        <v>204</v>
       </c>
       <c r="I173" t="s">
-        <v>260</v>
+        <v>219</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.2">
@@ -7593,7 +7500,7 @@
         <v>134</v>
       </c>
       <c r="C174" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D174" t="s">
         <v>12</v>
@@ -7616,19 +7523,19 @@
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
-        <v>264</v>
+        <v>223</v>
       </c>
       <c r="B175" s="5" t="s">
         <v>134</v>
       </c>
       <c r="C175" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D175" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>265</v>
+        <v>224</v>
       </c>
       <c r="F175">
         <v>2020</v>
@@ -7637,27 +7544,27 @@
         <v>2015</v>
       </c>
       <c r="H175" t="s">
-        <v>231</v>
+        <v>190</v>
       </c>
       <c r="I175" t="s">
-        <v>260</v>
+        <v>219</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A176" s="5" t="s">
-        <v>264</v>
+        <v>223</v>
       </c>
       <c r="B176" s="5" t="s">
         <v>134</v>
       </c>
       <c r="C176" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D176" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E176" s="3" t="s">
-        <v>266</v>
+        <v>225</v>
       </c>
       <c r="F176">
         <v>2019</v>
@@ -7666,10 +7573,10 @@
         <v>2015</v>
       </c>
       <c r="H176" t="s">
-        <v>243</v>
+        <v>202</v>
       </c>
       <c r="I176" t="s">
-        <v>260</v>
+        <v>219</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.2">
@@ -7680,7 +7587,7 @@
         <v>137</v>
       </c>
       <c r="C177" t="s">
-        <v>404</v>
+        <v>359</v>
       </c>
       <c r="D177" t="s">
         <v>22</v>
@@ -7700,19 +7607,19 @@
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="4" t="s">
-        <v>233</v>
+        <v>192</v>
       </c>
       <c r="B178" s="5" t="s">
         <v>137</v>
       </c>
       <c r="C178" t="s">
-        <v>404</v>
+        <v>359</v>
       </c>
       <c r="D178" t="s">
-        <v>234</v>
+        <v>193</v>
       </c>
       <c r="E178" t="s">
-        <v>236</v>
+        <v>195</v>
       </c>
       <c r="F178">
         <v>2013</v>
@@ -7721,7 +7628,7 @@
         <v>2005</v>
       </c>
       <c r="H178" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.2">
@@ -7732,13 +7639,13 @@
         <v>137</v>
       </c>
       <c r="C179" t="s">
-        <v>405</v>
+        <v>360</v>
       </c>
       <c r="D179" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E179" s="3" t="s">
-        <v>267</v>
+        <v>226</v>
       </c>
       <c r="F179">
         <v>2020</v>
@@ -7747,7 +7654,7 @@
         <v>2005</v>
       </c>
       <c r="H179" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.2">
@@ -7758,13 +7665,13 @@
         <v>137</v>
       </c>
       <c r="C180" t="s">
-        <v>405</v>
+        <v>360</v>
       </c>
       <c r="D180" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E180" s="3" t="s">
-        <v>268</v>
+        <v>227</v>
       </c>
       <c r="F180">
         <v>2020</v>
@@ -7773,7 +7680,7 @@
         <v>2005</v>
       </c>
       <c r="H180" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.2">
@@ -7784,13 +7691,13 @@
         <v>137</v>
       </c>
       <c r="C181" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D181" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E181" s="3" t="s">
-        <v>269</v>
+        <v>228</v>
       </c>
       <c r="F181" s="3">
         <v>2020</v>
@@ -7799,7 +7706,7 @@
         <v>2005</v>
       </c>
       <c r="H181" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.2">
@@ -7810,13 +7717,13 @@
         <v>137</v>
       </c>
       <c r="C182" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D182" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E182" s="3" t="s">
-        <v>271</v>
+        <v>230</v>
       </c>
       <c r="F182" s="3">
         <v>2020</v>
@@ -7825,7 +7732,7 @@
         <v>2005</v>
       </c>
       <c r="H182" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.2">
@@ -7836,7 +7743,7 @@
         <v>137</v>
       </c>
       <c r="C183" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D183" t="s">
         <v>12</v>
@@ -7862,7 +7769,7 @@
         <v>137</v>
       </c>
       <c r="C184" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D184" t="s">
         <v>12</v>
@@ -7888,7 +7795,7 @@
         <v>137</v>
       </c>
       <c r="C185" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D185" t="s">
         <v>12</v>
@@ -7914,7 +7821,7 @@
         <v>137</v>
       </c>
       <c r="C186" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D186" t="s">
         <v>12</v>
@@ -7940,7 +7847,7 @@
         <v>137</v>
       </c>
       <c r="C187" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D187" t="s">
         <v>12</v>
@@ -7966,7 +7873,7 @@
         <v>137</v>
       </c>
       <c r="C188" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D188" t="s">
         <v>12</v>
@@ -7992,7 +7899,7 @@
         <v>137</v>
       </c>
       <c r="C189" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D189" t="s">
         <v>12</v>
@@ -8018,7 +7925,7 @@
         <v>137</v>
       </c>
       <c r="C190" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D190" t="s">
         <v>12</v>
@@ -8044,7 +7951,7 @@
         <v>137</v>
       </c>
       <c r="C191" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D191" t="s">
         <v>12</v>
@@ -8070,7 +7977,7 @@
         <v>137</v>
       </c>
       <c r="C192" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D192" t="s">
         <v>12</v>
@@ -8093,10 +8000,10 @@
         <v>139</v>
       </c>
       <c r="B193" t="s">
-        <v>272</v>
+        <v>231</v>
       </c>
       <c r="C193" t="s">
-        <v>348</v>
+        <v>307</v>
       </c>
       <c r="D193" t="s">
         <v>12</v>
@@ -8122,13 +8029,13 @@
         <v>152</v>
       </c>
       <c r="C194" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D194" t="s">
         <v>12</v>
       </c>
       <c r="E194" s="3" t="s">
-        <v>305</v>
+        <v>264</v>
       </c>
       <c r="F194" s="3">
         <v>2020</v>
@@ -8137,7 +8044,7 @@
         <v>2009</v>
       </c>
       <c r="H194" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="195" spans="1:13" x14ac:dyDescent="0.2">
@@ -8145,16 +8052,16 @@
         <v>151</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>224</v>
+        <v>183</v>
       </c>
       <c r="C195" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D195" t="s">
         <v>12</v>
       </c>
       <c r="E195" s="3" t="s">
-        <v>306</v>
+        <v>265</v>
       </c>
       <c r="F195" s="3">
         <v>2020</v>
@@ -8163,7 +8070,7 @@
         <v>2009</v>
       </c>
       <c r="H195" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="196" spans="1:13" x14ac:dyDescent="0.2">
@@ -8174,13 +8081,13 @@
         <v>152</v>
       </c>
       <c r="C196" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D196" t="s">
         <v>12</v>
       </c>
       <c r="E196" s="3" t="s">
-        <v>307</v>
+        <v>266</v>
       </c>
       <c r="F196" s="3">
         <v>2012</v>
@@ -8189,7 +8096,7 @@
         <v>2009</v>
       </c>
       <c r="H196" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="197" spans="1:13" x14ac:dyDescent="0.2">
@@ -8197,10 +8104,10 @@
         <v>151</v>
       </c>
       <c r="B197" t="s">
-        <v>224</v>
+        <v>183</v>
       </c>
       <c r="C197" t="s">
-        <v>352</v>
+        <v>311</v>
       </c>
       <c r="D197" t="s">
         <v>12</v>
@@ -8226,7 +8133,7 @@
         <v>152</v>
       </c>
       <c r="C198" t="s">
-        <v>352</v>
+        <v>311</v>
       </c>
       <c r="D198" t="s">
         <v>12</v>
@@ -8252,7 +8159,7 @@
         <v>152</v>
       </c>
       <c r="C199" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D199" t="s">
         <v>12</v>
@@ -8278,7 +8185,7 @@
         <v>152</v>
       </c>
       <c r="C200" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D200" t="s">
         <v>12</v>
@@ -8304,7 +8211,7 @@
         <v>152</v>
       </c>
       <c r="C201" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D201" t="s">
         <v>12</v>
@@ -8330,7 +8237,7 @@
         <v>152</v>
       </c>
       <c r="C202" t="s">
-        <v>351</v>
+        <v>310</v>
       </c>
       <c r="D202" t="s">
         <v>12</v>
@@ -8359,16 +8266,16 @@
     </row>
     <row r="203" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A203" s="4" t="s">
-        <v>392</v>
+        <v>350</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>391</v>
+        <v>349</v>
       </c>
       <c r="C203" t="s">
-        <v>394</v>
+        <v>352</v>
       </c>
       <c r="D203" t="s">
-        <v>368</v>
+        <v>326</v>
       </c>
       <c r="E203">
         <v>93270</v>
@@ -8380,7 +8287,7 @@
         <v>2014</v>
       </c>
       <c r="H203" t="s">
-        <v>393</v>
+        <v>351</v>
       </c>
     </row>
     <row r="204" spans="1:13" x14ac:dyDescent="0.2">
@@ -8391,7 +8298,7 @@
         <v>160</v>
       </c>
       <c r="C204" t="s">
-        <v>394</v>
+        <v>352</v>
       </c>
       <c r="D204" t="s">
         <v>12</v>
@@ -8423,7 +8330,7 @@
         <v>36</v>
       </c>
       <c r="E205" t="s">
-        <v>418</v>
+        <v>373</v>
       </c>
       <c r="F205">
         <v>2015</v>
@@ -8443,7 +8350,7 @@
         <v>164</v>
       </c>
       <c r="C206" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D206" t="s">
         <v>12</v>
@@ -8469,7 +8376,7 @@
         <v>164</v>
       </c>
       <c r="C207" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D207" t="s">
         <v>12</v>
@@ -8495,7 +8402,7 @@
         <v>164</v>
       </c>
       <c r="C208" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D208" t="s">
         <v>12</v>
@@ -8521,13 +8428,13 @@
         <v>164</v>
       </c>
       <c r="C209" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D209" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E209" s="3" t="s">
-        <v>294</v>
+        <v>253</v>
       </c>
       <c r="F209" s="3">
         <v>2019</v>
@@ -8536,7 +8443,7 @@
         <v>2013</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.2">
@@ -8547,13 +8454,13 @@
         <v>164</v>
       </c>
       <c r="C210" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D210" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E210" s="3" t="s">
-        <v>295</v>
+        <v>254</v>
       </c>
       <c r="F210" s="3">
         <v>2019</v>
@@ -8562,7 +8469,7 @@
         <v>2013</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.2">
@@ -8573,13 +8480,13 @@
         <v>164</v>
       </c>
       <c r="C211" t="s">
-        <v>353</v>
+        <v>312</v>
       </c>
       <c r="D211" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E211" s="3" t="s">
-        <v>296</v>
+        <v>255</v>
       </c>
       <c r="F211" s="3">
         <v>2017</v>
@@ -8588,7 +8495,7 @@
         <v>2013</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>270</v>
+        <v>229</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.2">
@@ -8619,7 +8526,7 @@
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>293</v>
+        <v>252</v>
       </c>
       <c r="B213" t="s">
         <v>169</v>
@@ -8651,7 +8558,7 @@
         <v>173</v>
       </c>
       <c r="C214" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D214" t="s">
         <v>12</v>
@@ -8671,19 +8578,19 @@
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A215" s="4" t="s">
-        <v>273</v>
+        <v>232</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>274</v>
+        <v>233</v>
       </c>
       <c r="C215" t="s">
-        <v>350</v>
+        <v>309</v>
       </c>
       <c r="D215" t="s">
-        <v>252</v>
+        <v>211</v>
       </c>
       <c r="E215" s="3" t="s">
-        <v>275</v>
+        <v>234</v>
       </c>
       <c r="F215" s="3">
         <v>2024</v>
@@ -8692,24 +8599,24 @@
         <v>2018</v>
       </c>
       <c r="H215" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A216" s="4" t="s">
-        <v>365</v>
+        <v>387</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>397</v>
+        <v>355</v>
       </c>
       <c r="C216" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
       <c r="D216" t="s">
-        <v>361</v>
+        <v>320</v>
       </c>
       <c r="E216" s="7" t="s">
-        <v>398</v>
+        <v>356</v>
       </c>
       <c r="F216">
         <v>2020</v>
@@ -8718,483 +8625,34 @@
         <v>2020</v>
       </c>
       <c r="H216" t="s">
-        <v>235</v>
+        <v>194</v>
       </c>
       <c r="I216" t="s">
-        <v>421</v>
+        <v>375</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A217" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="B217" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="C217" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="D217" t="s">
-        <v>252</v>
-      </c>
-      <c r="E217" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="F217">
-        <v>2020</v>
-      </c>
-      <c r="G217">
-        <v>2020</v>
-      </c>
-      <c r="H217" t="s">
-        <v>282</v>
-      </c>
-      <c r="I217" t="s">
-        <v>421</v>
-      </c>
+      <c r="A217" s="4"/>
+      <c r="B217" s="9"/>
+      <c r="C217" s="3"/>
+      <c r="E217" s="3"/>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A218" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="B218" s="9" t="s">
-        <v>401</v>
-      </c>
-      <c r="C218" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="D218" t="s">
-        <v>252</v>
-      </c>
-      <c r="E218" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="F218">
-        <v>2019</v>
-      </c>
-      <c r="G218">
-        <v>2019</v>
-      </c>
-      <c r="H218" t="s">
-        <v>393</v>
-      </c>
-      <c r="I218" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A221" t="s">
-        <v>64</v>
-      </c>
-      <c r="B221" t="s">
-        <v>175</v>
-      </c>
-      <c r="C221">
-        <v>1</v>
-      </c>
-      <c r="D221" t="s">
-        <v>12</v>
-      </c>
-      <c r="E221" t="s">
-        <v>176</v>
-      </c>
-      <c r="F221">
-        <v>2023</v>
-      </c>
-      <c r="G221">
-        <v>2014</v>
-      </c>
-      <c r="H221" t="s">
-        <v>177</v>
-      </c>
-      <c r="I221" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A222" t="s">
-        <v>61</v>
-      </c>
-      <c r="B222" t="s">
-        <v>130</v>
-      </c>
-      <c r="C222">
-        <v>1</v>
-      </c>
-      <c r="D222" t="s">
-        <v>12</v>
-      </c>
-      <c r="E222" t="s">
-        <v>179</v>
-      </c>
-      <c r="F222">
-        <v>2024</v>
-      </c>
-      <c r="H222" t="s">
-        <v>177</v>
-      </c>
-      <c r="I222" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A223" t="s">
-        <v>129</v>
-      </c>
-      <c r="B223" t="s">
-        <v>181</v>
-      </c>
-      <c r="C223">
-        <v>1</v>
-      </c>
-      <c r="D223" t="s">
-        <v>12</v>
-      </c>
-      <c r="E223" t="s">
-        <v>182</v>
-      </c>
-      <c r="F223">
-        <v>2024</v>
-      </c>
-      <c r="H223" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
-        <v>119</v>
-      </c>
-      <c r="B224" t="s">
-        <v>184</v>
-      </c>
-      <c r="C224">
-        <v>1</v>
-      </c>
-      <c r="D224" t="s">
-        <v>12</v>
-      </c>
-      <c r="E224" t="s">
-        <v>185</v>
-      </c>
-      <c r="F224">
-        <v>2023</v>
-      </c>
-      <c r="H224" t="s">
-        <v>23</v>
-      </c>
-      <c r="I224" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A225" t="s">
-        <v>129</v>
-      </c>
-      <c r="B225" t="s">
-        <v>130</v>
-      </c>
-      <c r="C225">
-        <v>1</v>
-      </c>
-      <c r="D225" t="s">
-        <v>12</v>
-      </c>
-      <c r="E225" t="s">
-        <v>187</v>
-      </c>
-      <c r="F225">
-        <v>2023</v>
-      </c>
-      <c r="H225" t="s">
-        <v>23</v>
-      </c>
-      <c r="I225" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A226" t="s">
-        <v>119</v>
-      </c>
-      <c r="B226" t="s">
-        <v>130</v>
-      </c>
-      <c r="C226">
-        <v>1</v>
-      </c>
-      <c r="D226" t="s">
-        <v>12</v>
-      </c>
-      <c r="E226" t="s">
-        <v>189</v>
-      </c>
-      <c r="F226">
-        <v>2023</v>
-      </c>
-      <c r="H226" t="s">
-        <v>23</v>
-      </c>
-      <c r="I226" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A227" t="s">
-        <v>129</v>
-      </c>
-      <c r="B227" t="s">
-        <v>191</v>
-      </c>
-      <c r="C227">
-        <v>1</v>
-      </c>
-      <c r="D227" t="s">
-        <v>12</v>
-      </c>
-      <c r="E227" t="s">
-        <v>192</v>
-      </c>
-      <c r="F227">
-        <v>2024</v>
-      </c>
-      <c r="H227" t="s">
-        <v>193</v>
-      </c>
-      <c r="I227" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A228" t="s">
-        <v>119</v>
-      </c>
-      <c r="B228" t="s">
-        <v>120</v>
-      </c>
-      <c r="C228">
-        <v>1</v>
-      </c>
-      <c r="D228" t="s">
-        <v>12</v>
-      </c>
-      <c r="E228" t="s">
-        <v>195</v>
-      </c>
-      <c r="F228">
-        <v>2024</v>
-      </c>
-      <c r="H228" t="s">
-        <v>23</v>
-      </c>
-      <c r="I228" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A229" t="s">
-        <v>196</v>
-      </c>
-      <c r="B229" t="s">
-        <v>197</v>
-      </c>
-      <c r="C229">
-        <v>1</v>
-      </c>
-      <c r="D229" t="s">
-        <v>12</v>
-      </c>
-      <c r="E229" t="s">
-        <v>198</v>
-      </c>
-      <c r="F229">
-        <v>2024</v>
-      </c>
-      <c r="H229" t="s">
-        <v>23</v>
-      </c>
-      <c r="I229" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A230" t="s">
-        <v>200</v>
-      </c>
-      <c r="B230" t="s">
-        <v>201</v>
-      </c>
-      <c r="C230">
-        <v>1</v>
-      </c>
-      <c r="D230" t="s">
-        <v>12</v>
-      </c>
-      <c r="E230" t="s">
-        <v>202</v>
-      </c>
-      <c r="F230">
-        <v>2023</v>
-      </c>
-      <c r="H230" t="s">
-        <v>23</v>
-      </c>
-      <c r="I230" t="s">
-        <v>203</v>
-      </c>
+      <c r="A218" s="4"/>
+      <c r="B218" s="9"/>
+      <c r="C218" s="3"/>
+      <c r="E218" s="3"/>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A231" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="B231" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="C231" s="2">
-        <v>1</v>
-      </c>
-      <c r="D231" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E231" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F231" s="2">
-        <v>2023</v>
-      </c>
+      <c r="A231" s="1"/>
+      <c r="B231" s="2"/>
+      <c r="C231" s="2"/>
+      <c r="D231" s="2"/>
+      <c r="E231" s="2"/>
+      <c r="F231" s="2"/>
       <c r="G231" s="2"/>
-      <c r="H231" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I231" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A232" t="s">
-        <v>129</v>
-      </c>
-      <c r="B232" t="s">
-        <v>130</v>
-      </c>
-      <c r="C232" t="s">
-        <v>208</v>
-      </c>
-      <c r="D232" t="s">
-        <v>12</v>
-      </c>
-      <c r="E232" t="s">
-        <v>209</v>
-      </c>
-      <c r="F232">
-        <v>2023</v>
-      </c>
-      <c r="H232" t="s">
-        <v>23</v>
-      </c>
-      <c r="I232" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A233" t="s">
-        <v>107</v>
-      </c>
-      <c r="B233" t="s">
-        <v>211</v>
-      </c>
-      <c r="C233">
-        <v>1</v>
-      </c>
-      <c r="D233" t="s">
-        <v>12</v>
-      </c>
-      <c r="E233" t="s">
-        <v>212</v>
-      </c>
-      <c r="F233">
-        <v>2023</v>
-      </c>
-      <c r="H233" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A234" t="s">
-        <v>61</v>
-      </c>
-      <c r="B234" t="s">
-        <v>214</v>
-      </c>
-      <c r="C234">
-        <v>1</v>
-      </c>
-      <c r="D234" t="s">
-        <v>12</v>
-      </c>
-      <c r="E234" t="s">
-        <v>215</v>
-      </c>
-      <c r="F234">
-        <v>2024</v>
-      </c>
-      <c r="H234" t="s">
-        <v>23</v>
-      </c>
-      <c r="I234" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A235" t="s">
-        <v>126</v>
-      </c>
-      <c r="B235" t="s">
-        <v>188</v>
-      </c>
-      <c r="C235">
-        <v>1</v>
-      </c>
-      <c r="D235" t="s">
-        <v>12</v>
-      </c>
-      <c r="E235" t="s">
-        <v>217</v>
-      </c>
-      <c r="F235">
-        <v>2023</v>
-      </c>
-      <c r="H235" t="s">
-        <v>23</v>
-      </c>
-      <c r="I235" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A236" t="s">
-        <v>129</v>
-      </c>
-      <c r="B236" t="s">
-        <v>130</v>
-      </c>
-      <c r="C236" t="s">
-        <v>219</v>
-      </c>
-      <c r="D236" t="s">
-        <v>12</v>
-      </c>
-      <c r="E236" t="s">
-        <v>220</v>
-      </c>
-      <c r="F236">
-        <v>2023</v>
-      </c>
-      <c r="H236" t="s">
-        <v>37</v>
-      </c>
-      <c r="I236" t="s">
-        <v>221</v>
-      </c>
+      <c r="H231" s="2"/>
+      <c r="I231" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J218" xr:uid="{59979BBC-FF03-4FA8-9496-87716FB7753F}"/>

</xml_diff>